<commit_message>
Cleaned up variables to allow soft-coded tasks/function names
</commit_message>
<xml_diff>
--- a/EmployeeDatabase.xlsx
+++ b/EmployeeDatabase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myfir\Code and Repos\SchedulingCSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myfir\Repos\Git\SchedulingCSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4850DB9-2791-41D7-862B-223FE1A5E4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0614FC03-6940-4EEA-ACB4-711C831806F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28395" yWindow="-16440" windowWidth="29280" windowHeight="15960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,27 +64,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Task 1</t>
-  </si>
-  <si>
-    <t>Task 2</t>
-  </si>
-  <si>
-    <t>Task 3</t>
-  </si>
-  <si>
-    <t>Task 4</t>
-  </si>
-  <si>
-    <t>Task 5</t>
-  </si>
-  <si>
-    <t>Task 6</t>
-  </si>
-  <si>
-    <t>Task 7</t>
-  </si>
-  <si>
     <t>Emp 1</t>
   </si>
   <si>
@@ -476,6 +455,27 @@
   </si>
   <si>
     <t>Emp 131</t>
+  </si>
+  <si>
+    <t>Func 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Func 2 </t>
+  </si>
+  <si>
+    <t>Func 3</t>
+  </si>
+  <si>
+    <t>Func 4</t>
+  </si>
+  <si>
+    <t>Func 5</t>
+  </si>
+  <si>
+    <t>Func 6</t>
+  </si>
+  <si>
+    <t>Func 7</t>
   </si>
 </sst>
 </file>
@@ -529,9 +529,26 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="13">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -564,204 +581,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -777,28 +597,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7ED3E712-0A44-41FD-98FA-1CAB8F879D97}" name="Table1" displayName="Table1" ref="A1:I132" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7ED3E712-0A44-41FD-98FA-1CAB8F879D97}" name="Table1" displayName="Table1" ref="A1:I132" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:I132" xr:uid="{7ED3E712-0A44-41FD-98FA-1CAB8F879D97}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{5CF72A21-C9B7-4F44-A413-576B0941F8EF}" name="ID" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{56B1C5D0-1296-45A8-90FA-91B646964816}" name="Name" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{A43C75BF-F2A5-4CCD-97AF-C9E1F18BDFA8}" name="Task 1" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{A43C75BF-F2A5-4CCD-97AF-C9E1F18BDFA8}" name="Func 1" dataDxfId="8">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7CCD0307-EF1F-4B2D-B4F5-131F6F4BF1AC}" name="Task 2" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{21D045C2-E09E-45DB-8D8D-C124A9055F89}" name="Task 3" dataDxfId="6">
+    <tableColumn id="4" xr3:uid="{7CCD0307-EF1F-4B2D-B4F5-131F6F4BF1AC}" name="Func 2 " dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{21D045C2-E09E-45DB-8D8D-C124A9055F89}" name="Func 3" dataDxfId="6">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{BB53661E-385E-4FF6-930C-B0553875370D}" name="Task 4" dataDxfId="5">
+    <tableColumn id="6" xr3:uid="{BB53661E-385E-4FF6-930C-B0553875370D}" name="Func 4" dataDxfId="5">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{BF6EAB39-8BB5-45A4-9785-A2BFA30D3003}" name="Task 5" dataDxfId="4">
+    <tableColumn id="7" xr3:uid="{BF6EAB39-8BB5-45A4-9785-A2BFA30D3003}" name="Func 5" dataDxfId="4">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{5CBDFEC2-7AB0-4AA5-8ABF-ED7EAD93D7D1}" name="Task 6" dataDxfId="3">
+    <tableColumn id="8" xr3:uid="{5CBDFEC2-7AB0-4AA5-8ABF-ED7EAD93D7D1}" name="Func 6" dataDxfId="3">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{ACBBA126-0BE8-4062-BF15-1D931227F88F}" name="Task 7" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{ACBBA126-0BE8-4062-BF15-1D931227F88F}" name="Func 7" dataDxfId="2">
       <calculatedColumnFormula>FALSE</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1070,9 +890,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1080,34 +900,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="C2" s="1" t="b">
         <f>TRUE</f>
         <v>1</v>
@@ -1137,12 +957,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C3" s="1" t="b">
         <f>TRUE</f>
@@ -1173,12 +993,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="b">
         <f>TRUE</f>
@@ -1209,12 +1029,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C5" s="1" t="b">
         <f>TRUE</f>
@@ -1245,12 +1065,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1" t="b">
         <f>TRUE</f>
@@ -1281,12 +1101,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C7" s="1" t="b">
         <f>TRUE</f>
@@ -1317,12 +1137,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C8" s="1" t="b">
         <f>TRUE</f>
@@ -1353,12 +1173,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1" t="b">
         <f>TRUE</f>
@@ -1389,12 +1209,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C10" s="1" t="b">
         <f>TRUE</f>
@@ -1425,12 +1245,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C11" s="1" t="b">
         <f>TRUE</f>
@@ -1461,12 +1281,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C12" s="1" t="b">
         <f>TRUE</f>
@@ -1497,12 +1317,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C13" s="1" t="b">
         <f>TRUE</f>
@@ -1533,12 +1353,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C14" s="1" t="b">
         <f>TRUE</f>
@@ -1569,12 +1389,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C15" s="1" t="b">
         <f>TRUE</f>
@@ -1605,12 +1425,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C16" s="1" t="b">
         <f>TRUE</f>
@@ -1641,12 +1461,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C17" s="1" t="b">
         <f>TRUE</f>
@@ -1677,12 +1497,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C18" s="1" t="b">
         <f>TRUE</f>
@@ -1713,12 +1533,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C19" s="1" t="b">
         <f>TRUE</f>
@@ -1749,12 +1569,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="b">
         <f>TRUE</f>
@@ -1785,12 +1605,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C21" s="1" t="b">
         <f>TRUE</f>
@@ -1821,12 +1641,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C22" s="1" t="b">
         <f>TRUE</f>
@@ -1857,12 +1677,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C23" s="1" t="b">
         <f>TRUE</f>
@@ -1893,12 +1713,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C24" s="1" t="b">
         <f>TRUE</f>
@@ -1929,12 +1749,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C25" s="1" t="b">
         <f>TRUE</f>
@@ -1965,12 +1785,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C26" s="1" t="b">
         <f>TRUE</f>
@@ -2001,12 +1821,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C27" s="1" t="b">
         <f>TRUE</f>
@@ -2037,12 +1857,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C28" s="1" t="b">
         <f>TRUE</f>
@@ -2073,12 +1893,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C29" s="1" t="b">
         <f>TRUE</f>
@@ -2109,12 +1929,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C30" s="1" t="b">
         <f>TRUE</f>
@@ -2145,12 +1965,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C31" s="1" t="b">
         <f>TRUE</f>
@@ -2181,12 +2001,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" s="1">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C32" s="1" t="b">
         <f>TRUE</f>
@@ -2217,12 +2037,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" s="1">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C33" s="1" t="b">
         <f>TRUE</f>
@@ -2253,12 +2073,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" s="1">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C34" s="1" t="b">
         <f>TRUE</f>
@@ -2289,12 +2109,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" s="1">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C35" s="1" t="b">
         <f>TRUE</f>
@@ -2325,12 +2145,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" s="1">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C36" s="1" t="b">
         <f>TRUE</f>
@@ -2361,12 +2181,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" s="1">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C37" s="1" t="b">
         <f>TRUE</f>
@@ -2397,12 +2217,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" s="1">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C38" s="1" t="b">
         <f>TRUE</f>
@@ -2433,12 +2253,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" s="1">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C39" s="1" t="b">
         <f>TRUE</f>
@@ -2469,12 +2289,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" s="1">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C40" s="1" t="b">
         <f>TRUE</f>
@@ -2505,12 +2325,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" s="1">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C41" s="1" t="b">
         <f>TRUE</f>
@@ -2541,12 +2361,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" s="1">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C42" s="1" t="b">
         <f>TRUE</f>
@@ -2577,12 +2397,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A43" s="1">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C43" s="1" t="b">
         <f>TRUE</f>
@@ -2613,12 +2433,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" s="1">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C44" s="1" t="b">
         <f>TRUE</f>
@@ -2649,12 +2469,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" s="1">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C45" s="1" t="b">
         <f>TRUE</f>
@@ -2685,12 +2505,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" s="1">
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C46" s="1" t="b">
         <f>TRUE</f>
@@ -2721,12 +2541,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A47" s="1">
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C47" s="1" t="b">
         <f>TRUE</f>
@@ -2757,12 +2577,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" s="1">
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C48" s="1" t="b">
         <f>TRUE</f>
@@ -2793,12 +2613,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" s="1">
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C49" s="1" t="b">
         <f>TRUE</f>
@@ -2829,12 +2649,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" s="1">
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C50" s="1" t="b">
         <f>TRUE</f>
@@ -2865,12 +2685,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" s="1">
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C51" s="1" t="b">
         <f>TRUE</f>
@@ -2901,12 +2721,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" s="1">
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C52" s="1" t="b">
         <f>TRUE</f>
@@ -2937,12 +2757,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" s="1">
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C53" s="1" t="b">
         <f>TRUE</f>
@@ -2973,12 +2793,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" s="1">
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C54" s="1" t="b">
         <f>TRUE</f>
@@ -3009,12 +2829,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" s="1">
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C55" s="1" t="b">
         <f>TRUE</f>
@@ -3045,12 +2865,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" s="1">
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C56" s="1" t="b">
         <f>TRUE</f>
@@ -3081,12 +2901,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" s="1">
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C57" s="1" t="b">
         <f>TRUE</f>
@@ -3117,12 +2937,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" s="1">
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C58" s="1" t="b">
         <f>TRUE</f>
@@ -3153,12 +2973,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" s="1">
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C59" s="1" t="b">
         <f>TRUE</f>
@@ -3189,12 +3009,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" s="1">
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C60" s="1" t="b">
         <f>TRUE</f>
@@ -3225,12 +3045,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" s="1">
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C61" s="1" t="b">
         <f>TRUE</f>
@@ -3261,12 +3081,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A62" s="1">
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C62" s="1" t="b">
         <f>TRUE</f>
@@ -3297,12 +3117,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" s="1">
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C63" s="1" t="b">
         <f>TRUE</f>
@@ -3333,12 +3153,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" s="1">
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C64" s="1" t="b">
         <f>TRUE</f>
@@ -3369,12 +3189,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A65" s="1">
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C65" s="1" t="b">
         <f>TRUE</f>
@@ -3405,12 +3225,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A66" s="1">
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C66" s="1" t="b">
         <f>TRUE</f>
@@ -3441,12 +3261,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A67" s="1">
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C67" s="1" t="b">
         <f>TRUE</f>
@@ -3477,12 +3297,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A68" s="1">
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C68" s="1" t="b">
         <f>TRUE</f>
@@ -3513,12 +3333,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A69" s="1">
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C69" s="1" t="b">
         <f>TRUE</f>
@@ -3549,12 +3369,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A70" s="1">
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C70" s="1" t="b">
         <f>TRUE</f>
@@ -3585,12 +3405,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A71" s="1">
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C71" s="1" t="b">
         <f>TRUE</f>
@@ -3621,12 +3441,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A72" s="1">
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C72" s="1" t="b">
         <f>TRUE</f>
@@ -3657,12 +3477,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A73" s="1">
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C73" s="1" t="b">
         <f>TRUE</f>
@@ -3693,12 +3513,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A74" s="1">
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C74" s="1" t="b">
         <f>TRUE</f>
@@ -3729,12 +3549,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A75" s="1">
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C75" s="1" t="b">
         <f>TRUE</f>
@@ -3765,12 +3585,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A76" s="1">
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C76" s="1" t="b">
         <f>TRUE</f>
@@ -3801,12 +3621,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A77" s="1">
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C77" s="1" t="b">
         <f>TRUE</f>
@@ -3837,12 +3657,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A78" s="1">
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C78" s="1" t="b">
         <f>TRUE</f>
@@ -3873,12 +3693,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A79" s="1">
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C79" s="1" t="b">
         <f>TRUE</f>
@@ -3909,12 +3729,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A80" s="1">
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C80" s="1" t="b">
         <f>TRUE</f>
@@ -3945,12 +3765,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A81" s="1">
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C81" s="1" t="b">
         <f>TRUE</f>
@@ -3981,12 +3801,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A82" s="1">
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C82" s="1" t="b">
         <f>TRUE</f>
@@ -4017,12 +3837,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A83" s="1">
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C83" s="1" t="b">
         <f>TRUE</f>
@@ -4053,12 +3873,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A84" s="1">
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C84" s="1" t="b">
         <f>TRUE</f>
@@ -4089,12 +3909,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A85" s="1">
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C85" s="1" t="b">
         <f>TRUE</f>
@@ -4125,12 +3945,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A86" s="1">
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C86" s="1" t="b">
         <f>TRUE</f>
@@ -4161,12 +3981,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A87" s="1">
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C87" s="1" t="b">
         <f>TRUE</f>
@@ -4197,12 +4017,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A88" s="1">
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C88" s="1" t="b">
         <f>TRUE</f>
@@ -4233,12 +4053,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A89" s="1">
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="C89" s="1" t="b">
         <f>TRUE</f>
@@ -4269,12 +4089,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A90" s="1">
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C90" s="1" t="b">
         <f>TRUE</f>
@@ -4305,12 +4125,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A91" s="1">
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C91" s="1" t="b">
         <f>TRUE</f>
@@ -4341,12 +4161,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A92" s="1">
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C92" s="1" t="b">
         <f>TRUE</f>
@@ -4354,15 +4174,15 @@
       </c>
       <c r="D92" s="1" t="b">
         <f t="shared" ref="D92:D124" ca="1" si="0">IF(RAND() &gt; 0.4, TRUE, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E92" s="1" t="b">
         <f t="shared" ref="E92:E124" ca="1" si="1">IF(RAND() &gt; 0.7, TRUE, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92" s="1" t="b">
         <f t="shared" ref="F92:G124" ca="1" si="2">IF(RAND() &gt; 0.8, TRUE, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G92" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4377,12 +4197,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A93" s="1">
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="C93" s="1" t="b">
         <f>TRUE</f>
@@ -4410,15 +4230,15 @@
       </c>
       <c r="I93" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A94" s="1">
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C94" s="1" t="b">
         <f>TRUE</f>
@@ -4434,7 +4254,7 @@
       </c>
       <c r="F94" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4449,12 +4269,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A95" s="1">
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C95" s="1" t="b">
         <f>TRUE</f>
@@ -4466,7 +4286,7 @@
       </c>
       <c r="E95" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F95" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4474,7 +4294,7 @@
       </c>
       <c r="G95" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -4485,12 +4305,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A96" s="1">
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C96" s="1" t="b">
         <f>TRUE</f>
@@ -4502,7 +4322,7 @@
       </c>
       <c r="E96" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F96" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4510,7 +4330,7 @@
       </c>
       <c r="G96" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H96" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -4521,12 +4341,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A97" s="1">
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C97" s="1" t="b">
         <f>TRUE</f>
@@ -4557,12 +4377,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A98" s="1">
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C98" s="1" t="b">
         <f>TRUE</f>
@@ -4570,7 +4390,7 @@
       </c>
       <c r="D98" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E98" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -4578,11 +4398,11 @@
       </c>
       <c r="F98" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G98" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H98" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -4593,12 +4413,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A99" s="1">
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C99" s="1" t="b">
         <f>TRUE</f>
@@ -4610,7 +4430,7 @@
       </c>
       <c r="E99" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F99" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4626,15 +4446,15 @@
       </c>
       <c r="I99" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A100" s="1">
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C100" s="1" t="b">
         <f>TRUE</f>
@@ -4642,7 +4462,7 @@
       </c>
       <c r="D100" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E100" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -4650,7 +4470,7 @@
       </c>
       <c r="F100" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G100" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4665,12 +4485,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A101" s="1">
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C101" s="1" t="b">
         <f>TRUE</f>
@@ -4678,11 +4498,11 @@
       </c>
       <c r="D101" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E101" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F101" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4701,12 +4521,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A102" s="1">
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C102" s="1" t="b">
         <f>TRUE</f>
@@ -4714,11 +4534,11 @@
       </c>
       <c r="D102" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E102" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F102" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4737,12 +4557,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A103" s="1">
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C103" s="1" t="b">
         <f>TRUE</f>
@@ -4750,11 +4570,11 @@
       </c>
       <c r="D103" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E103" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F103" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4773,12 +4593,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A104" s="1">
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C104" s="1" t="b">
         <f>TRUE</f>
@@ -4794,7 +4614,7 @@
       </c>
       <c r="F104" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G104" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4802,19 +4622,19 @@
       </c>
       <c r="H104" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I104" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A105" s="1">
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C105" s="1" t="b">
         <f>TRUE</f>
@@ -4826,11 +4646,11 @@
       </c>
       <c r="E105" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F105" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4838,19 +4658,19 @@
       </c>
       <c r="H105" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I105" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A106" s="1">
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C106" s="1" t="b">
         <f>TRUE</f>
@@ -4870,23 +4690,23 @@
       </c>
       <c r="G106" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H106" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I106" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A107" s="1">
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C107" s="1" t="b">
         <f>TRUE</f>
@@ -4894,19 +4714,19 @@
       </c>
       <c r="D107" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E107" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F107" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G107" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H107" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -4917,12 +4737,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A108" s="1">
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C108" s="1" t="b">
         <f>TRUE</f>
@@ -4938,7 +4758,7 @@
       </c>
       <c r="F108" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -4953,12 +4773,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A109" s="1">
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C109" s="1" t="b">
         <f>TRUE</f>
@@ -4974,27 +4794,27 @@
       </c>
       <c r="F109" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G109" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H109" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I109" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A110" s="1">
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C110" s="1" t="b">
         <f>TRUE</f>
@@ -5002,7 +4822,7 @@
       </c>
       <c r="D110" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E110" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -5010,11 +4830,11 @@
       </c>
       <c r="F110" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H110" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -5025,12 +4845,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A111" s="1">
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C111" s="1" t="b">
         <f>TRUE</f>
@@ -5058,15 +4878,15 @@
       </c>
       <c r="I111" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A112" s="1">
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C112" s="1" t="b">
         <f>TRUE</f>
@@ -5074,11 +4894,11 @@
       </c>
       <c r="D112" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E112" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F112" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5086,7 +4906,7 @@
       </c>
       <c r="G112" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H112" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -5097,12 +4917,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A113" s="1">
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C113" s="1" t="b">
         <f>TRUE</f>
@@ -5118,7 +4938,7 @@
       </c>
       <c r="F113" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5133,12 +4953,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A114" s="1">
         <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C114" s="1" t="b">
         <f>TRUE</f>
@@ -5146,11 +4966,11 @@
       </c>
       <c r="D114" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E114" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F114" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5169,12 +4989,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A115" s="1">
         <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C115" s="1" t="b">
         <f>TRUE</f>
@@ -5186,7 +5006,7 @@
       </c>
       <c r="E115" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F115" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5205,12 +5025,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A116" s="1">
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C116" s="1" t="b">
         <f>TRUE</f>
@@ -5222,7 +5042,7 @@
       </c>
       <c r="E116" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F116" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5241,12 +5061,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A117" s="1">
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C117" s="1" t="b">
         <f>TRUE</f>
@@ -5262,11 +5082,11 @@
       </c>
       <c r="F117" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G117" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H117" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -5277,12 +5097,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A118" s="1">
         <v>117</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C118" s="1" t="b">
         <f>TRUE</f>
@@ -5298,7 +5118,7 @@
       </c>
       <c r="F118" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G118" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5313,12 +5133,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A119" s="1">
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C119" s="1" t="b">
         <f>TRUE</f>
@@ -5330,11 +5150,11 @@
       </c>
       <c r="E119" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F119" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G119" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5349,12 +5169,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A120" s="1">
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C120" s="1" t="b">
         <f>TRUE</f>
@@ -5370,11 +5190,11 @@
       </c>
       <c r="F120" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G120" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H120" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -5382,15 +5202,15 @@
       </c>
       <c r="I120" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A121" s="1">
         <v>120</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C121" s="1" t="b">
         <f>TRUE</f>
@@ -5402,7 +5222,7 @@
       </c>
       <c r="E121" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F121" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5421,12 +5241,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A122" s="1">
         <v>121</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C122" s="1" t="b">
         <f>TRUE</f>
@@ -5446,7 +5266,7 @@
       </c>
       <c r="G122" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
@@ -5457,12 +5277,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A123" s="1">
         <v>122</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C123" s="1" t="b">
         <f>TRUE</f>
@@ -5474,11 +5294,11 @@
       </c>
       <c r="E123" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F123" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G123" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5490,15 +5310,15 @@
       </c>
       <c r="I123" s="1" t="b">
         <f t="shared" ca="1" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A124" s="1">
         <v>123</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C124" s="1" t="b">
         <f>TRUE</f>
@@ -5506,15 +5326,15 @@
       </c>
       <c r="D124" s="1" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E124" s="1" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F124" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124" s="1" t="b">
         <f t="shared" ca="1" si="2"/>
@@ -5529,12 +5349,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A125" s="1">
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C125" s="1" t="b">
         <f>FALSE</f>
@@ -5565,12 +5385,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A126" s="1">
         <v>125</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C126" s="1" t="b">
         <f>FALSE</f>
@@ -5601,12 +5421,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A127" s="1">
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C127" s="1" t="b">
         <f>FALSE</f>
@@ -5637,12 +5457,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A128" s="1">
         <v>127</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C128" s="1" t="b">
         <f>FALSE</f>
@@ -5673,12 +5493,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A129" s="1">
         <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C129" s="1" t="b">
         <f>FALSE</f>
@@ -5709,12 +5529,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A130" s="1">
         <v>129</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C130" s="1" t="b">
         <f>FALSE</f>
@@ -5745,12 +5565,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A131" s="1">
         <v>130</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C131" s="1" t="b">
         <f>TRUE</f>
@@ -5781,12 +5601,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A132" s="1">
         <v>131</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C132" s="1" t="b">
         <f>FALSE</f>
@@ -5820,11 +5640,11 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C2:I132">
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>FALSE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="1" operator="equal">
-      <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>